<commit_message>
Generate reference baselines from exhibition history
</commit_message>
<xml_diff>
--- a/templates/ilmin-report-input-template.xlsx
+++ b/templates/ilmin-report-input-template.xlsx
@@ -3,9 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="core" sheetId="1" r:id="rId1"/>
-    <sheet name="reference-groups" sheetId="2" r:id="rId2"/>
-    <sheet name="selected-feedback" sheetId="3" r:id="rId3"/>
-    <sheet name="data-quality" sheetId="4" r:id="rId4"/>
+    <sheet name="reference-exhibitions" sheetId="2" r:id="rId2"/>
+    <sheet name="reference-groups" sheetId="3" r:id="rId3"/>
+    <sheet name="selected-feedback" sheetId="4" r:id="rId4"/>
+    <sheet name="data-quality" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -177,22 +178,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">period</t>
+          <t xml:space="preserve">exhibition</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">start</t>
+          <t xml:space="preserve">type</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-06-13</t>
+          <t xml:space="preserve">정기 기획전</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">YYYY-MM-DD</t>
+          <t xml:space="preserve">정기 기획전, 특별전, 기타 중 선택</t>
         </is>
       </c>
     </row>
@@ -204,12 +205,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">end</t>
+          <t xml:space="preserve">start</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-08-17</t>
+          <t xml:space="preserve">2025-06-13</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -226,56 +227,56 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">display</t>
+          <t xml:space="preserve">end</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025.06.13 - 2025.08.17</t>
+          <t xml:space="preserve">2025-08-17</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">report display</t>
+          <t xml:space="preserve">YYYY-MM-DD</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">exhibition</t>
+          <t xml:space="preserve">period</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">scope_note</t>
+          <t xml:space="preserve">display</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">엑셀 입력 템플릿에서 변환한 v4.3 데모입니다. 관객 후기는 전체 여론이 아니라 선별 입력값입니다.</t>
+          <t xml:space="preserve">2025.06.13 - 2025.08.17</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">report display</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">narrative</t>
+          <t xml:space="preserve">exhibition</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">theme_and_content</t>
+          <t xml:space="preserve">scope_note</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">이 전시는 색채 경험과 공간 몰입을 중심으로 관객의 전시 체류와 반응을 관찰하기 위한 v4.3 샘플입니다. 실제 보고서에서는 전시 기획 의도와 전시 주제에 관한 서술을 이 항목에 입력합니다.</t>
+          <t xml:space="preserve">엑셀 입력 템플릿에서 변환한 v4.3 데모입니다. 관객 후기는 전체 여론이 아니라 선별 입력값입니다.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -292,12 +293,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">composition_note</t>
+          <t xml:space="preserve">theme_and_content</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">전시 구성 항목에는 전시실별 구성·작품 수·공간 연출·연계 프로그램 운영 내역을 입력합니다. 현재 샘플은 프로그램 참여 지표를 중심으로 구성됩니다.</t>
+          <t xml:space="preserve">이 전시는 색채 경험과 공간 몰입을 중심으로 관객의 전시 체류와 반응을 관찰하기 위한 v4.3 샘플입니다. 실제 보고서에서는 전시 기획 의도와 전시 주제에 관한 서술을 이 항목에 입력합니다.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -314,25 +315,15 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">evaluation_note</t>
+          <t xml:space="preserve">composition_note</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">평가 및 개선방안 항목은 성공/실패 판정이 아니라 수치상 특이점</t>
+          <t xml:space="preserve">전시 구성 항목에는 전시실별 구성·작품 수·공간 연출·연계 프로그램 운영 내역을 입력합니다. 현재 샘플은 프로그램 참여 지표를 중심으로 구성됩니다.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 관객 반응</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 데이터 검증 필요 사항을 후속 참고사항으로 정리합니다.</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -341,20 +332,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">audience</t>
+          <t xml:space="preserve">narrative</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">total_visitors</t>
+          <t xml:space="preserve">evaluation_note</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">15200</t>
+          <t xml:space="preserve">평가 및 개선방안 항목은 성공/실패 판정이 아니라 수치상 특이점</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 관객 반응</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 데이터 검증 필요 사항을 후속 참고사항으로 정리합니다.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -368,12 +369,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">operating_days</t>
+          <t xml:space="preserve">total_visitors</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">66</t>
+          <t xml:space="preserve">15200</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -390,17 +391,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">daily_visitors</t>
+          <t xml:space="preserve">operating_days</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">230</t>
+          <t xml:space="preserve">66</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank allowed if operating_days exists</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -412,17 +413,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">paid_visitors</t>
+          <t xml:space="preserve">daily_visitors</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">8907</t>
+          <t xml:space="preserve">230</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">blank allowed if operating_days exists</t>
         </is>
       </c>
     </row>
@@ -434,12 +435,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">free_visitors</t>
+          <t xml:space="preserve">paid_visitors</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">6293</t>
+          <t xml:space="preserve">8907</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -451,17 +452,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">budget</t>
+          <t xml:space="preserve">audience</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">total_budget</t>
+          <t xml:space="preserve">free_visitors</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">210000000</t>
+          <t xml:space="preserve">6293</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -478,12 +479,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">income</t>
+          <t xml:space="preserve">total_budget</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">210000000</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -495,17 +496,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">programs</t>
+          <t xml:space="preserve">budget</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">count</t>
+          <t xml:space="preserve">income</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -522,12 +523,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">sessions</t>
+          <t xml:space="preserve">count</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">65</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -544,12 +545,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">participants</t>
+          <t xml:space="preserve">sessions</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">548</t>
+          <t xml:space="preserve">65</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -566,12 +567,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">participation_rate</t>
+          <t xml:space="preserve">participants</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.6</t>
+          <t xml:space="preserve">548</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -583,17 +584,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">publicity</t>
+          <t xml:space="preserve">programs</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">press_mentions</t>
+          <t xml:space="preserve">participation_rate</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">32</t>
+          <t xml:space="preserve">3.6</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -610,12 +611,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">sns_posts</t>
+          <t xml:space="preserve">press_mentions</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">24</t>
+          <t xml:space="preserve">32</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -627,17 +628,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">membership</t>
+          <t xml:space="preserve">publicity</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">memberships_sold</t>
+          <t xml:space="preserve">sns_posts</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -654,12 +655,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">memberships_sold</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">v4.3 샘플에서는 멤버십 분석을 생성하지 않습니다.</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -671,20 +672,42 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t xml:space="preserve">membership</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">note</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v4.3 샘플에서는 멤버십 분석을 생성하지 않습니다.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t xml:space="preserve">brief_metrics</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t xml:space="preserve">ids</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t xml:space="preserve">total_visitors,daily_visitors,total_budget,cost_per_visitor,program_participants,press_mentions</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -695,6 +718,1301 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="23" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">total_visitors</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">operating_days</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">daily_visitors</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">total_budget</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">income</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">cost_per_visitor</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">program_participants</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">press_mentions</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">paid_audience_ratio</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9200</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">58</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">138000000</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">27000000</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">760</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">86</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 02</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10100</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">63</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">142000000</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31000000</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">820</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">88</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8700</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">55</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">132000000</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25000000</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">710</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">84</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 04</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9600</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">149000000</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33000000</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">89</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">68</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">155000000</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36000000</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">950</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7900</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120000000</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21000000</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">650</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">82</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 07</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9300</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">59</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">136000000</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28000000</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">790</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">86</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regular-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 정기 기획전 08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정기 기획전</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10500</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">66</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">148000000</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34000000</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">870</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">88</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">special-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 특별전 01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">특별전</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18200</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">320000000</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">62000000</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1020</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">special-02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 특별전 02</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">특별전</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21400</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">380000000</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81000000</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1180</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">55</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">special-03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 특별전 03</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">특별전</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16800</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">65</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">295000000</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">57000000</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">940</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">44</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">69</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">special-04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 특별전 04</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">특별전</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24000</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">410000000</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93000000</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1320</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">special-05</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 특별전 05</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">특별전</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19700</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">76</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">350000000</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">76000000</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1110</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">special-06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 특별전 06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">특별전</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15300</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">280000000</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">51000000</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">880</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">68</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">other-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 기타 전시 01</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5200</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70000000</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9000000</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">320</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">63</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">other-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 기타 전시 02</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6100</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">82000000</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11000000</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">410</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">66</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">other-03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 기타 전시 03</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4300</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">65000000</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7000000</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">280</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">58</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">other-04</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 기타 전시 04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7400</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92000000</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14000000</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">470</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">67</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -885,7 +2203,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1060,7 +2378,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>

</xml_diff>

<commit_message>
Select fixed and recommended director metrics
</commit_message>
<xml_diff>
--- a/templates/ilmin-report-input-template.xlsx
+++ b/templates/ilmin-report-input-template.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">35600000</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">total_visitors,daily_visitors,total_budget,cost_per_visitor,program_participants,press_mentions</t>
+          <t xml:space="preserve">total_visitors,daily_visitors,total_budget,total_income,cost_per_visitor,auto</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">

</xml_diff>

<commit_message>
Fix director metric card inputs
</commit_message>
<xml_diff>
--- a/templates/ilmin-report-input-template.xlsx
+++ b/templates/ilmin-report-input-template.xlsx
@@ -474,17 +474,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">budget</t>
+          <t xml:space="preserve">audience</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">total_budget</t>
+          <t xml:space="preserve">group_visitors</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">210000000</t>
+          <t xml:space="preserve">1216</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -501,12 +501,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">income</t>
+          <t xml:space="preserve">total_budget</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">35600000</t>
+          <t xml:space="preserve">210000000</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -518,17 +518,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">programs</t>
+          <t xml:space="preserve">budget</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">count</t>
+          <t xml:space="preserve">execution_rate</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">92.4</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -540,17 +540,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">programs</t>
+          <t xml:space="preserve">budget</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">sessions</t>
+          <t xml:space="preserve">income</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">65</t>
+          <t xml:space="preserve">35600000</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -567,12 +567,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">participants</t>
+          <t xml:space="preserve">count</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">548</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">participation_rate</t>
+          <t xml:space="preserve">sessions</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.6</t>
+          <t xml:space="preserve">65</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -606,17 +606,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">publicity</t>
+          <t xml:space="preserve">programs</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">press_mentions</t>
+          <t xml:space="preserve">participants</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">32</t>
+          <t xml:space="preserve">548</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -628,17 +628,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">publicity</t>
+          <t xml:space="preserve">programs</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">sns_posts</t>
+          <t xml:space="preserve">participation_rate</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">24</t>
+          <t xml:space="preserve">3.6</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -650,17 +650,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">membership</t>
+          <t xml:space="preserve">publicity</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">memberships_sold</t>
+          <t xml:space="preserve">press_mentions</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">32</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -672,17 +672,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">membership</t>
+          <t xml:space="preserve">publicity</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">sns_posts</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">v4.3 샘플에서는 멤버십 분석을 생성하지 않습니다.</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -694,20 +694,86 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t xml:space="preserve">publicity</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sns_feedback_total</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">186</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">membership</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">memberships_sold</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">membership</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">note</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v4.3 샘플에서는 멤버십 분석을 생성하지 않습니다.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t xml:space="preserve">brief_metrics</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t xml:space="preserve">ids</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">total_visitors,daily_visitors,total_budget,total_income,program_participants,program_participation_rate,press_mentions,sns_feedback,cost_per_visitor,auto</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">total_visitors,daily_visitors,total_budget,budget_execution_rate,total_income,cost_per_visitor,paid_audience_ratio,group_audience_ratio,program_sessions,program_participants,press_mentions,sns_feedback</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Refine director metric strip comparisons
</commit_message>
<xml_diff>
--- a/templates/ilmin-report-input-template.xlsx
+++ b/templates/ilmin-report-input-template.xlsx
@@ -793,12 +793,16 @@
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="23" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="23" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -839,30 +843,50 @@
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">execution_rate</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">income</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">cost_per_visitor</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">group_visitors</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">program_sessions</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">program_participants</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">press_mentions</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="O1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">paid_audience_ratio</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sns_feedback_total</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">note</t>
         </is>
@@ -906,30 +930,50 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t xml:space="preserve">88.6</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t xml:space="preserve">27000000</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">620</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t xml:space="preserve">760</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">29</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t xml:space="preserve">86</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10006</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -973,30 +1017,50 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t xml:space="preserve">91.2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t xml:space="preserve">31000000</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">710</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">58</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t xml:space="preserve">820</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">30</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t xml:space="preserve">88</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">126796</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1040,30 +1104,50 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t xml:space="preserve">86.5</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t xml:space="preserve">25000000</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">540</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">44</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t xml:space="preserve">710</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t xml:space="preserve">26</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t xml:space="preserve">84</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">151278</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1107,30 +1191,50 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t xml:space="preserve">94.1</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t xml:space="preserve">33000000</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">650</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">63</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t xml:space="preserve">900</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t xml:space="preserve">32</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t xml:space="preserve">89</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">131977</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1174,30 +1278,50 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t xml:space="preserve">90.7</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t xml:space="preserve">36000000</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">860</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t xml:space="preserve">950</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t xml:space="preserve">34</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t xml:space="preserve">87</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="P6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">140171</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1241,30 +1365,50 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t xml:space="preserve">84.3</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t xml:space="preserve">21000000</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">430</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t xml:space="preserve">650</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t xml:space="preserve">23</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t xml:space="preserve">82</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">152389</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1308,30 +1452,50 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t xml:space="preserve">89.8</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t xml:space="preserve">28000000</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">610</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">50</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t xml:space="preserve">790</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t xml:space="preserve">28</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t xml:space="preserve">86</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">156645</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1375,30 +1539,50 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t xml:space="preserve">92.4</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t xml:space="preserve">34000000</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">760</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">62</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t xml:space="preserve">870</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t xml:space="preserve">31</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">88</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="P9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">144986</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1442,30 +1626,50 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t xml:space="preserve">93.0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t xml:space="preserve">62000000</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">980</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t xml:space="preserve">1020</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t xml:space="preserve">48</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t xml:space="preserve">71</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="P10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">392724</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1509,30 +1713,50 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t xml:space="preserve">95.2</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t xml:space="preserve">81000000</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1260</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">82</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t xml:space="preserve">1180</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t xml:space="preserve">55</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t xml:space="preserve">75</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">400400</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1576,30 +1800,50 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t xml:space="preserve">90.5</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t xml:space="preserve">57000000</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">880</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">64</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t xml:space="preserve">940</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t xml:space="preserve">44</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t xml:space="preserve">69</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="P12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10364</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1643,30 +1887,50 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
+          <t xml:space="preserve">97.6</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
           <t xml:space="preserve">93000000</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1420</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
           <t xml:space="preserve">1320</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t xml:space="preserve">61</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t xml:space="preserve">77</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="P13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330529</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1710,30 +1974,50 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t xml:space="preserve">94.4</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
           <t xml:space="preserve">76000000</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1140</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">79</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t xml:space="preserve">1110</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t xml:space="preserve">52</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t xml:space="preserve">74</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="P14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1057337</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1777,30 +2061,50 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t xml:space="preserve">88.7</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
           <t xml:space="preserve">51000000</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">760</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">58</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t xml:space="preserve">880</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t xml:space="preserve">39</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t xml:space="preserve">68</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="P15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">689513</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1844,30 +2148,50 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t xml:space="preserve">81.5</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t xml:space="preserve">9000000</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">280</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t xml:space="preserve">320</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t xml:space="preserve">12</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t xml:space="preserve">63</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="P16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52000</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1911,30 +2235,50 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
+          <t xml:space="preserve">85.7</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
           <t xml:space="preserve">11000000</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">350</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t xml:space="preserve">410</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t xml:space="preserve">16</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t xml:space="preserve">66</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="P17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61000</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1978,30 +2322,50 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
+          <t xml:space="preserve">79.9</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t xml:space="preserve">7000000</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">190</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
           <t xml:space="preserve">280</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t xml:space="preserve">9</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t xml:space="preserve">58</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="P18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43000</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2045,30 +2409,50 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
+          <t xml:space="preserve">87.1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t xml:space="preserve">14000000</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">430</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
           <t xml:space="preserve">470</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t xml:space="preserve">67</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="P19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74000</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2088,10 +2472,14 @@
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
-    <col min="11" max="11" width="27" customWidth="1"/>
+    <col min="8" max="8" width="29" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="28" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="27" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2132,22 +2520,42 @@
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">budget_execution_rate_avg</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">cost_per_visitor_avg</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">group_audience_ratio_avg</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">program_sessions_avg</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">program_participants_avg</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">press_mentions_avg</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">paid_audience_ratio_avg</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">sns_feedback_avg</t>
         </is>
       </c>
     </row>
@@ -2189,22 +2597,42 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t xml:space="preserve">89.7</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t xml:space="preserve">20000</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.9</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">55</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t xml:space="preserve">807.6</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t xml:space="preserve">28.9</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">86.6</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">126781</t>
         </is>
       </c>
     </row>
@@ -2260,6 +2688,26 @@
         </is>
       </c>
       <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>